<commit_message>
Publish the build 55 Variables and Calculations workbook as its own download
Co-Authored-By: Alisha Kanwar <alisha.kanwar@ppischool.in>
</commit_message>
<xml_diff>
--- a/Variables and Calculations.xlsx
+++ b/Variables and Calculations.xlsx
@@ -11,9 +11,12 @@
     <sheet name="MW Capacity" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Plant Master" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Constants" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="RM Nature" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FG Master" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TB Master" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RM Technology Costs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="RM Plant Costs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="RM Constants" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="RM Nature" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FG Master" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TB Master" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -641,72 +644,205 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>RM Nature     one row per raw-material code: its nature, the group it belongs to</t>
+          <t>RM Technology Costs   only the Cost INR/Wp inputs for the Module and Cell component</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              (Module or Cell, which is what draws the two blocks on the RM page)</t>
+          <t xml:space="preserve">              rows. Dates run across the top; add a new dated column when a cost</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              and its BOM standard quantity. Paste your rows under the headings.</t>
+          <t xml:space="preserve">              changes. Blank means carry the last value forward; 0 is an intentional</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              zero. Total Module and Total Cell are calculated in Power BI.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>FG Master     one row per finished-goods code and the technology it is.</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>RM Plant Costs   separate Cost INR/Wp inputs for 1900 and 1902. They can differ for</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TB Master     one row per GL account: what it is, and the plant it belongs to. The</t>
+          <t xml:space="preserve">              the same item. Dates and carry-forward work exactly as above.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">              GL number is the only key the trial balance and this sheet share, so</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              an account with no plant here is an account the report cannot place -</t>
+          <t>RM Constants   Module and Cell production constants plus the 1900 and 1902 plant</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              write 1902, 1900 or 1905 against it, or the plant's name.</t>
+          <t xml:space="preserve">              variables (1900 Dholera Module = 5, 1902 Jaipur = 8 initially). Add a</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              dated column when one changes; never type derived totals, inventory</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">              values, per-day costs or Days on these sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>RM Nature     one row per raw-material code: its nature, the group it belongs to</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              (Module or Cell, which is what draws the two blocks on the RM page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              and its BOM standard quantity. Paste your rows under the headings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>FG Master     one row per finished-goods code and the technology it is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>TB Master     one row per GL account: what it is, and the plant it belongs to. The</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              GL number is the only key the trial balance and this sheet share, so</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              an account with no plant here is an account the report cannot place -</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              write 1902, 1900 or 1905 against it, or the plant's name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t>One habit to keep: close this workbook before refreshing the report.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>GL Account Number</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>GL Account Description</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Plant</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Sort Order</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Plant takes 1902, 1900 or 1905 - or the plant's name. An inventory GL with this column empty is one the trial balance cannot place, which is what Checks reports as an unresolved profit centre.</t>
         </is>
       </c>
     </row>
@@ -1203,6 +1339,550 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Plant Group</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Only type externally supplied Cost INR/Wp values. Add a new dated column to the right when a value changes; blank carries forward and 0 is intentional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cell Cost</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Cell Cost-G12R</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Glass</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Packing Material-M</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>POE</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Wafer</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2.11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Paste</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1.87</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Gases</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Chemical</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Packing Material</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Plant</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>1900 and 1902 costs are independent. Add a new dated column when a value changes; do not type inventory, per-day cost or Days here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cell Cost</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Glass</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Packing Material-M</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>POE</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Cell Cost</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Cell Cost-G12R</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Glass</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Packing Material-M</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>POE</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Constant Name</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Only the four externally supplied constants belong here. Add a new dated column when one changes; blank carries the prior value forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Module Production Constant</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Cell Production Constant</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1900 Plant Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1902 Plant Variable</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1263,7 +1943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1309,58 +1989,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>GL Account Number</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>GL Account Description</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Nature</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Plant</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Sort Order</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Plant takes 1902, 1900 or 1905 - or the plant's name. An inventory GL with this column empty is one the trial balance cannot place, which is what Checks reports as an unresolved profit centre.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
TB Master starter sheet carries profit centre columns
Co-Authored-By: Alisha Kanwar <alisha.kanwar@ppischool.in>
</commit_message>
<xml_diff>
--- a/Variables and Calculations.xlsx
+++ b/Variables and Calculations.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -757,36 +757,43 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TB Master     one row per GL account: what it is, and the plant it belongs to. The</t>
+          <t>TB Master     one row per GL account and profit centre: what the account is, the</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              GL number is the only key the trial balance and this sheet share, so</t>
+          <t xml:space="preserve">              profit centre it was posted to, and the plant that pair belongs to.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              an account with no plant here is an account the report cannot place -</t>
+          <t xml:space="preserve">              GL number and profit centre are the keys the trial balance shares with</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">              write 1902, 1900 or 1905 against it, or the plant's name.</t>
+          <t xml:space="preserve">              this sheet, so a pair with no plant is money the report cannot place -</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              write 1902, 1900 or 1905 in Plant, and its name in 'at'.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>One habit to keep: close this workbook before refreshing the report.</t>
         </is>
@@ -803,15 +810,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -827,22 +837,37 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Profit Centre</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Profit Centre Description</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Nature</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Plant</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Sort Order</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Plant takes 1902, 1900 or 1905 - or the plant's name. An inventory GL with this column empty is one the trial balance cannot place, which is what Checks reports as an unresolved profit centre.</t>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>One row per GL account and profit centre pair, which is how the trial balance splits one account across plants. Plant takes 1902, 1900 or 1905 and 'at' is that plant's name. An inventory GL with Plant empty is one the trial balance cannot place, which is what Checks reports as an unresolved profit centre.</t>
         </is>
       </c>
     </row>

</xml_diff>